<commit_message>
Add Email column to EMAIL_LIST.xlsx
</commit_message>
<xml_diff>
--- a/EMAIL_LIST.xlsx
+++ b/EMAIL_LIST.xlsx
@@ -397,27 +397,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:D1"/>
   <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="1" max="1" width="40.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="30.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>Email</v>
+      </c>
+      <c r="B1" t="str">
         <v>Date of Entering</v>
       </c>
-      <c r="B1" t="str">
+      <c r="C1" t="str">
         <v>Time of Entering</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>Subscribed for Daily Article</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>